<commit_message>
data: 台股 財報估值(179檔, 自算PER) 20260625
</commit_message>
<xml_diff>
--- a/data/20260625_台股財報估值.xlsx
+++ b/data/20260625_台股財報估值.xlsx
@@ -23293,7 +23293,11 @@
           <t>兆豐金</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
       <c r="D243" t="inlineStr">
         <is>
           <t>2026-03-31</t>
@@ -23375,7 +23379,11 @@
           <t>合庫金</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr"/>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
       <c r="D244" t="inlineStr">
         <is>
           <t>2026-03-31</t>
@@ -44309,7 +44317,11 @@
           <t>兆豐金</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
       <c r="D243" t="n">
         <v>0</v>
       </c>
@@ -44385,7 +44397,11 @@
           <t>合庫金</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr"/>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
       <c r="D244" t="n">
         <v>0</v>
       </c>

</xml_diff>